<commit_message>
prints and new excel
</commit_message>
<xml_diff>
--- a/Entries HBC Premier Elite 2024.xlsx
+++ b/Entries HBC Premier Elite 2024.xlsx
@@ -27399,2032 +27399,2032 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
-      <c r="B2" s="65" t="inlineStr">
+      <c r="B2" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="C2" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="D2" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="E2" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="F2" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="G2" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="H2" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="I2" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="J2" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="K2" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="L2" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="M2" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="N2" s="51" t="inlineStr">
+        <is>
+          <t>MD V - 1</t>
+        </is>
+      </c>
+      <c r="O2" s="55" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="P2" s="64" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="Q2" s="59" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="R2" s="56" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="S2" s="49" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="T2" s="49" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="U2" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="V2" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="W2" s="62" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="X2" s="57" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="Y2" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="Z2" s="51" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AA2" s="53" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="AB2" s="55" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="AC2" s="60" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="AD2" s="61" t="inlineStr">
+        <is>
+          <t>WD B - 2</t>
+        </is>
+      </c>
+      <c r="AE2" s="63" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="AF2" s="62" t="inlineStr">
+        <is>
+          <t>WD A - 2</t>
+        </is>
+      </c>
+      <c r="AG2" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 4</t>
+        </is>
+      </c>
+      <c r="AH2" s="54" t="inlineStr">
+        <is>
+          <t>WD V - 2</t>
+        </is>
+      </c>
+      <c r="AI2" s="55" t="inlineStr">
+        <is>
+          <t>MS V - 3</t>
+        </is>
+      </c>
+      <c r="AJ2" s="55" t="inlineStr">
+        <is>
+          <t>MS V - 3</t>
+        </is>
+      </c>
+      <c r="AK2" s="59" t="inlineStr">
+        <is>
+          <t>XD B - 4</t>
+        </is>
+      </c>
+      <c r="AL2" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 5</t>
+        </is>
+      </c>
+      <c r="AM2" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 4</t>
+        </is>
+      </c>
+      <c r="AN2" s="49" t="inlineStr">
+        <is>
+          <t>XD V - 4</t>
+        </is>
+      </c>
+      <c r="AO2" s="55" t="inlineStr">
+        <is>
+          <t>MS V - 4</t>
+        </is>
+      </c>
+      <c r="AP2" s="55" t="inlineStr">
+        <is>
+          <t>MS V - 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="C3" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="D3" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="E3" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="F3" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="G3" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="H3" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="I3" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="J3" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="K3" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="L3" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="M3" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="N3" s="49" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="O3" s="55" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="P3" s="64" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="Q3" s="59" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="R3" s="56" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="S3" s="49" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="T3" s="49" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="U3" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="V3" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="W3" s="62" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="X3" s="57" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="Y3" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="Z3" s="51" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AA3" s="53" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="AB3" s="55" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="AC3" s="60" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="AD3" s="61" t="inlineStr">
+        <is>
+          <t>WD B - 2</t>
+        </is>
+      </c>
+      <c r="AE3" s="63" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="AF3" s="62" t="inlineStr">
+        <is>
+          <t>WD A - 2</t>
+        </is>
+      </c>
+      <c r="AG3" s="57" t="inlineStr">
+        <is>
+          <t>WS A - 2</t>
+        </is>
+      </c>
+      <c r="AH3" s="54" t="inlineStr">
+        <is>
+          <t>WD V - 2</t>
+        </is>
+      </c>
+      <c r="AI3" s="55" t="inlineStr">
+        <is>
+          <t>MS V - 3</t>
+        </is>
+      </c>
+      <c r="AJ3" s="55" t="inlineStr">
+        <is>
+          <t>MS V - 3</t>
+        </is>
+      </c>
+      <c r="AK3" s="59" t="inlineStr">
+        <is>
+          <t>XD B - 4</t>
+        </is>
+      </c>
+      <c r="AL3" s="63" t="inlineStr">
+        <is>
+          <t>WS B - 3</t>
+        </is>
+      </c>
+      <c r="AM3" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 4</t>
+        </is>
+      </c>
+      <c r="AN3" s="49" t="inlineStr">
+        <is>
+          <t>XD V - 4</t>
+        </is>
+      </c>
+      <c r="AO3" s="53" t="inlineStr">
+        <is>
+          <t>WS V - 4</t>
+        </is>
+      </c>
+      <c r="AP3" s="55" t="inlineStr">
+        <is>
+          <t>MS V - 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="C4" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="D4" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="E4" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="F4" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="G4" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="H4" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="I4" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="J4" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="K4" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="L4" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="M4" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="N4" s="49" t="inlineStr">
+        <is>
+          <t>XD V - 1</t>
+        </is>
+      </c>
+      <c r="O4" s="55" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="P4" s="64" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="Q4" s="59" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="R4" s="56" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="S4" s="49" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="T4" s="49" t="inlineStr">
+        <is>
+          <t>XD V - 3</t>
+        </is>
+      </c>
+      <c r="U4" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="V4" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="W4" s="62" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="X4" s="57" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="Y4" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="Z4" s="51" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AA4" s="53" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="AB4" s="55" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="AC4" s="60" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="AD4" s="59" t="inlineStr">
+        <is>
+          <t>XD B - 3</t>
+        </is>
+      </c>
+      <c r="AE4" s="63" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="AF4" s="62" t="inlineStr">
+        <is>
+          <t>WD A - 2</t>
+        </is>
+      </c>
+      <c r="AG4" s="57" t="inlineStr">
+        <is>
+          <t>WS A - 2</t>
+        </is>
+      </c>
+      <c r="AH4" s="54" t="inlineStr">
+        <is>
+          <t>WD V - 2</t>
+        </is>
+      </c>
+      <c r="AI4" s="53" t="inlineStr">
+        <is>
+          <t>WS V - 3</t>
+        </is>
+      </c>
+      <c r="AJ4" s="64" t="inlineStr">
+        <is>
+          <t>MD C - 4</t>
+        </is>
+      </c>
+      <c r="AK4" s="59" t="inlineStr">
+        <is>
+          <t>XD B - 5</t>
+        </is>
+      </c>
+      <c r="AL4" s="63" t="inlineStr">
+        <is>
+          <t>WS B - 3</t>
+        </is>
+      </c>
+      <c r="AM4" s="62" t="inlineStr">
+        <is>
+          <t>WD A - 3</t>
+        </is>
+      </c>
+      <c r="AN4" s="49" t="inlineStr">
+        <is>
+          <t>XD V - 5</t>
+        </is>
+      </c>
+      <c r="AO4" s="53" t="inlineStr">
+        <is>
+          <t>WS V - 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="C5" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="D5" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="E5" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="F5" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="G5" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="H5" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="I5" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="J5" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="K5" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="L5" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="M5" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="N5" s="56" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="O5" s="55" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="P5" s="65" t="inlineStr">
         <is>
           <t>XD C - 1</t>
         </is>
       </c>
-      <c r="C2" s="66" t="inlineStr">
+      <c r="Q5" s="59" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="R5" s="56" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="S5" s="49" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="T5" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="U5" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="V5" s="63" t="inlineStr">
+        <is>
+          <t>WS B - 1</t>
+        </is>
+      </c>
+      <c r="W5" s="62" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="X5" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="Y5" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="Z5" s="51" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AA5" s="53" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="AB5" s="55" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="AC5" s="64" t="inlineStr">
+        <is>
+          <t>MD C - 3</t>
+        </is>
+      </c>
+      <c r="AD5" s="59" t="inlineStr">
+        <is>
+          <t>XD B - 3</t>
+        </is>
+      </c>
+      <c r="AE5" s="63" t="inlineStr">
+        <is>
+          <t>WS B - 2</t>
+        </is>
+      </c>
+      <c r="AF5" s="56" t="inlineStr">
+        <is>
+          <t>XD A - 3</t>
+        </is>
+      </c>
+      <c r="AG5" s="57" t="inlineStr">
+        <is>
+          <t>WS A - 2</t>
+        </is>
+      </c>
+      <c r="AH5" s="54" t="inlineStr">
+        <is>
+          <t>WD V - 2</t>
+        </is>
+      </c>
+      <c r="AI5" s="53" t="inlineStr">
+        <is>
+          <t>WS V - 3</t>
+        </is>
+      </c>
+      <c r="AJ5" s="64" t="inlineStr">
+        <is>
+          <t>MD C - 4</t>
+        </is>
+      </c>
+      <c r="AK5" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 5</t>
+        </is>
+      </c>
+      <c r="AL5" s="63" t="inlineStr">
+        <is>
+          <t>WS B - 4</t>
+        </is>
+      </c>
+      <c r="AM5" s="62" t="inlineStr">
+        <is>
+          <t>WD A - 3</t>
+        </is>
+      </c>
+      <c r="AN5" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 5</t>
+        </is>
+      </c>
+      <c r="AO5" s="53" t="inlineStr">
+        <is>
+          <t>WS V - 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="C6" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="D6" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="E6" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="F6" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="G6" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="H6" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="I6" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="J6" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="K6" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="L6" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="M6" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="N6" s="56" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="O6" s="55" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="P6" s="65" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="Q6" s="64" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="R6" s="56" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="S6" s="49" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="T6" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="U6" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="V6" s="63" t="inlineStr">
+        <is>
+          <t>WS B - 1</t>
+        </is>
+      </c>
+      <c r="W6" s="62" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="X6" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="Y6" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="Z6" s="51" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AA6" s="53" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="AB6" s="55" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="AC6" s="64" t="inlineStr">
+        <is>
+          <t>MD C - 3</t>
+        </is>
+      </c>
+      <c r="AD6" s="59" t="inlineStr">
+        <is>
+          <t>XD B - 3</t>
+        </is>
+      </c>
+      <c r="AE6" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="AF6" s="56" t="inlineStr">
+        <is>
+          <t>XD A - 3</t>
+        </is>
+      </c>
+      <c r="AG6" s="57" t="inlineStr">
+        <is>
+          <t>WS A - 2</t>
+        </is>
+      </c>
+      <c r="AH6" s="49" t="inlineStr">
+        <is>
+          <t>XD V - 3</t>
+        </is>
+      </c>
+      <c r="AI6" s="53" t="inlineStr">
+        <is>
+          <t>WS V - 3</t>
+        </is>
+      </c>
+      <c r="AJ6" s="66" t="inlineStr">
+        <is>
+          <t>WD C - 2</t>
+        </is>
+      </c>
+      <c r="AK6" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 5</t>
+        </is>
+      </c>
+      <c r="AL6" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 4</t>
+        </is>
+      </c>
+      <c r="AM6" s="62" t="inlineStr">
+        <is>
+          <t>WD A - 4</t>
+        </is>
+      </c>
+      <c r="AN6" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 5</t>
+        </is>
+      </c>
+      <c r="AO6" s="51" t="inlineStr">
+        <is>
+          <t>MD V - 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="C7" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="D7" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="E7" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="F7" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="G7" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="H7" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="I7" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="J7" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="K7" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="L7" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="M7" s="64" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="N7" s="56" t="inlineStr">
+        <is>
+          <t>XD A - 1</t>
+        </is>
+      </c>
+      <c r="O7" s="55" t="inlineStr">
+        <is>
+          <t>MS V - 1</t>
+        </is>
+      </c>
+      <c r="P7" s="65" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="Q7" s="64" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="R7" s="59" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="S7" s="49" t="inlineStr">
+        <is>
+          <t>XD V - 2</t>
+        </is>
+      </c>
+      <c r="T7" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="U7" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="V7" s="63" t="inlineStr">
+        <is>
+          <t>WS B - 1</t>
+        </is>
+      </c>
+      <c r="W7" s="62" t="inlineStr">
+        <is>
+          <t>WD A - 1</t>
+        </is>
+      </c>
+      <c r="X7" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="Y7" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="Z7" s="51" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AA7" s="53" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="AB7" s="55" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="AC7" s="64" t="inlineStr">
+        <is>
+          <t>MD C - 3</t>
+        </is>
+      </c>
+      <c r="AD7" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 4</t>
+        </is>
+      </c>
+      <c r="AE7" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="AF7" s="56" t="inlineStr">
+        <is>
+          <t>XD A - 3</t>
+        </is>
+      </c>
+      <c r="AG7" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 3</t>
+        </is>
+      </c>
+      <c r="AH7" s="49" t="inlineStr">
+        <is>
+          <t>XD V - 3</t>
+        </is>
+      </c>
+      <c r="AI7" s="53" t="inlineStr">
+        <is>
+          <t>WS V - 3</t>
+        </is>
+      </c>
+      <c r="AJ7" s="66" t="inlineStr">
+        <is>
+          <t>WD C - 2</t>
+        </is>
+      </c>
+      <c r="AK7" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 6</t>
+        </is>
+      </c>
+      <c r="AL7" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 4</t>
+        </is>
+      </c>
+      <c r="AM7" s="56" t="inlineStr">
+        <is>
+          <t>XD A - 4</t>
+        </is>
+      </c>
+      <c r="AN7" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 6</t>
+        </is>
+      </c>
+      <c r="AO7" s="51" t="inlineStr">
+        <is>
+          <t>MD V - 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="C8" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="D8" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="E8" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="F8" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="G8" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="H8" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="I8" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="J8" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="K8" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="L8" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="M8" s="64" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="N8" s="59" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="O8" s="53" t="inlineStr">
+        <is>
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="P8" s="65" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="Q8" s="64" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="R8" s="59" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="S8" s="56" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="T8" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="U8" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 2</t>
+        </is>
+      </c>
+      <c r="V8" s="63" t="inlineStr">
+        <is>
+          <t>WS B - 1</t>
+        </is>
+      </c>
+      <c r="W8" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="X8" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="Y8" s="57" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="Z8" s="54" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="AA8" s="53" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="AB8" s="55" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="AC8" s="66" t="inlineStr">
         <is>
           <t>WD C - 1</t>
         </is>
       </c>
-      <c r="D2" s="64" t="inlineStr">
+      <c r="AD8" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 4</t>
+        </is>
+      </c>
+      <c r="AE8" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="AF8" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 4</t>
+        </is>
+      </c>
+      <c r="AG8" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 3</t>
+        </is>
+      </c>
+      <c r="AH8" s="49" t="inlineStr">
+        <is>
+          <t>XD V - 3</t>
+        </is>
+      </c>
+      <c r="AI8" s="51" t="inlineStr">
+        <is>
+          <t>MD V - 3</t>
+        </is>
+      </c>
+      <c r="AJ8" s="66" t="inlineStr">
+        <is>
+          <t>WD C - 3</t>
+        </is>
+      </c>
+      <c r="AK8" s="60" t="inlineStr">
+        <is>
+          <t>WS C - 3</t>
+        </is>
+      </c>
+      <c r="AL8" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 5</t>
+        </is>
+      </c>
+      <c r="AM8" s="56" t="inlineStr">
+        <is>
+          <t>XD A - 4</t>
+        </is>
+      </c>
+      <c r="AN8" s="57" t="inlineStr">
+        <is>
+          <t>WS A - 3</t>
+        </is>
+      </c>
+      <c r="AO8" s="51" t="inlineStr">
+        <is>
+          <t>MD V - 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="C9" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="D9" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="E9" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="F9" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="G9" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="H9" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="I9" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 2</t>
+        </is>
+      </c>
+      <c r="J9" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="K9" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="L9" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="M9" s="64" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="N9" s="59" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="O9" s="53" t="inlineStr">
+        <is>
+          <t>WS V - 1</t>
+        </is>
+      </c>
+      <c r="P9" s="65" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="Q9" s="64" t="inlineStr">
         <is>
           <t>MD C - 2</t>
         </is>
       </c>
-      <c r="E2" s="64" t="inlineStr">
+      <c r="R9" s="59" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="S9" s="56" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="T9" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="U9" s="61" t="inlineStr">
+        <is>
+          <t>WD B - 1</t>
+        </is>
+      </c>
+      <c r="V9" s="63" t="inlineStr">
+        <is>
+          <t>WS B - 1</t>
+        </is>
+      </c>
+      <c r="W9" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="X9" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="Y9" s="57" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="Z9" s="54" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="AA9" s="53" t="inlineStr">
+        <is>
+          <t>WS V - 2</t>
+        </is>
+      </c>
+      <c r="AB9" s="55" t="inlineStr">
+        <is>
+          <t>MS V - 2</t>
+        </is>
+      </c>
+      <c r="AC9" s="66" t="inlineStr">
+        <is>
+          <t>WD C - 1</t>
+        </is>
+      </c>
+      <c r="AD9" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 4</t>
+        </is>
+      </c>
+      <c r="AE9" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 3</t>
+        </is>
+      </c>
+      <c r="AF9" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 4</t>
+        </is>
+      </c>
+      <c r="AG9" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 3</t>
+        </is>
+      </c>
+      <c r="AH9" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 4</t>
+        </is>
+      </c>
+      <c r="AI9" s="51" t="inlineStr">
+        <is>
+          <t>MD V - 3</t>
+        </is>
+      </c>
+      <c r="AJ9" s="65" t="inlineStr">
+        <is>
+          <t>XD C - 3</t>
+        </is>
+      </c>
+      <c r="AK9" s="60" t="inlineStr">
+        <is>
+          <t>WS C - 3</t>
+        </is>
+      </c>
+      <c r="AL9" s="61" t="inlineStr">
+        <is>
+          <t>WD B - 3</t>
+        </is>
+      </c>
+      <c r="AM9" s="56" t="inlineStr">
+        <is>
+          <t>XD A - 5</t>
+        </is>
+      </c>
+      <c r="AN9" s="57" t="inlineStr">
+        <is>
+          <t>WS A - 3</t>
+        </is>
+      </c>
+      <c r="AO9" s="54" t="inlineStr">
+        <is>
+          <t>WD V - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="C10" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="D10" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="E10" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 1</t>
+        </is>
+      </c>
+      <c r="F10" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="G10" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="H10" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="I10" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="J10" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="K10" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="L10" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="M10" s="64" t="inlineStr">
         <is>
           <t>MD C - 1</t>
         </is>
       </c>
-      <c r="F2" s="60" t="inlineStr">
+      <c r="N10" s="59" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="O10" s="65" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="P10" s="65" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="Q10" s="64" t="inlineStr">
+        <is>
+          <t>MD C - 2</t>
+        </is>
+      </c>
+      <c r="R10" s="59" t="inlineStr">
+        <is>
+          <t>XD B - 2</t>
+        </is>
+      </c>
+      <c r="S10" s="56" t="inlineStr">
+        <is>
+          <t>XD A - 2</t>
+        </is>
+      </c>
+      <c r="T10" s="60" t="inlineStr">
         <is>
           <t>WS C - 1</t>
         </is>
       </c>
-      <c r="G2" s="47" t="inlineStr">
+      <c r="U10" s="47" t="inlineStr">
         <is>
           <t>MS C - 3</t>
         </is>
       </c>
-      <c r="H2" s="47" t="inlineStr">
+      <c r="V10" s="63" t="inlineStr">
+        <is>
+          <t>WS B - 1</t>
+        </is>
+      </c>
+      <c r="W10" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="X10" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="Y10" s="57" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="Z10" s="54" t="inlineStr">
+        <is>
+          <t>WD V - 1</t>
+        </is>
+      </c>
+      <c r="AA10" s="51" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AB10" s="65" t="inlineStr">
+        <is>
+          <t>XD C - 2</t>
+        </is>
+      </c>
+      <c r="AC10" s="66" t="inlineStr">
+        <is>
+          <t>WD C - 1</t>
+        </is>
+      </c>
+      <c r="AD10" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 4</t>
+        </is>
+      </c>
+      <c r="AE10" s="61" t="inlineStr">
+        <is>
+          <t>WD B - 2</t>
+        </is>
+      </c>
+      <c r="AF10" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 4</t>
+        </is>
+      </c>
+      <c r="AG10" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 3</t>
+        </is>
+      </c>
+      <c r="AH10" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 4</t>
+        </is>
+      </c>
+      <c r="AI10" s="51" t="inlineStr">
+        <is>
+          <t>MD V - 3</t>
+        </is>
+      </c>
+      <c r="AJ10" s="65" t="inlineStr">
+        <is>
+          <t>XD C - 3</t>
+        </is>
+      </c>
+      <c r="AK10" s="60" t="inlineStr">
+        <is>
+          <t>WS C - 4</t>
+        </is>
+      </c>
+      <c r="AL10" s="61" t="inlineStr">
+        <is>
+          <t>WD B - 3</t>
+        </is>
+      </c>
+      <c r="AM10" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 5</t>
+        </is>
+      </c>
+      <c r="AN10" s="57" t="inlineStr">
+        <is>
+          <t>WS A - 4</t>
+        </is>
+      </c>
+      <c r="AO10" s="54" t="inlineStr">
+        <is>
+          <t>WD V - 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 1</t>
+        </is>
+      </c>
+      <c r="C11" s="47" t="inlineStr">
         <is>
           <t>MS C - 2</t>
         </is>
       </c>
-      <c r="I2" s="47" t="inlineStr">
+      <c r="D11" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 1</t>
+        </is>
+      </c>
+      <c r="E11" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="F11" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 2</t>
+        </is>
+      </c>
+      <c r="G11" s="47" t="inlineStr">
         <is>
           <t>MS C - 2</t>
         </is>
       </c>
-      <c r="J2" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="K2" s="59" t="inlineStr">
+      <c r="H11" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 2</t>
+        </is>
+      </c>
+      <c r="I11" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="J11" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="K11" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 1</t>
+        </is>
+      </c>
+      <c r="L11" s="58" t="inlineStr">
+        <is>
+          <t>MD B - 1</t>
+        </is>
+      </c>
+      <c r="M11" s="64" t="inlineStr">
+        <is>
+          <t>MD C - 1</t>
+        </is>
+      </c>
+      <c r="N11" s="59" t="inlineStr">
+        <is>
+          <t>XD B - 1</t>
+        </is>
+      </c>
+      <c r="O11" s="65" t="inlineStr">
+        <is>
+          <t>XD C - 1</t>
+        </is>
+      </c>
+      <c r="P11" s="65" t="inlineStr">
+        <is>
+          <t>XD C - 2</t>
+        </is>
+      </c>
+      <c r="Q11" s="64" t="inlineStr">
+        <is>
+          <t>MD C - 3</t>
+        </is>
+      </c>
+      <c r="R11" s="59" t="inlineStr">
         <is>
           <t>XD B - 3</t>
         </is>
       </c>
-      <c r="L2" s="59" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="M2" s="61" t="inlineStr">
+      <c r="S11" s="56" t="inlineStr">
+        <is>
+          <t>XD A - 3</t>
+        </is>
+      </c>
+      <c r="T11" s="60" t="inlineStr">
+        <is>
+          <t>WS C - 1</t>
+        </is>
+      </c>
+      <c r="U11" s="47" t="inlineStr">
+        <is>
+          <t>MS C - 3</t>
+        </is>
+      </c>
+      <c r="V11" s="63" t="inlineStr">
+        <is>
+          <t>WS B - 1</t>
+        </is>
+      </c>
+      <c r="W11" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 3</t>
+        </is>
+      </c>
+      <c r="X11" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 2</t>
+        </is>
+      </c>
+      <c r="Y11" s="57" t="inlineStr">
+        <is>
+          <t>WS A - 1</t>
+        </is>
+      </c>
+      <c r="Z11" s="52" t="inlineStr">
+        <is>
+          <t>MS A - 3</t>
+        </is>
+      </c>
+      <c r="AA11" s="51" t="inlineStr">
+        <is>
+          <t>MD V - 2</t>
+        </is>
+      </c>
+      <c r="AB11" s="65" t="inlineStr">
+        <is>
+          <t>XD C - 2</t>
+        </is>
+      </c>
+      <c r="AC11" s="65" t="inlineStr">
+        <is>
+          <t>XD C - 2</t>
+        </is>
+      </c>
+      <c r="AD11" s="60" t="inlineStr">
+        <is>
+          <t>WS C - 2</t>
+        </is>
+      </c>
+      <c r="AE11" s="61" t="inlineStr">
         <is>
           <t>WD B - 2</t>
         </is>
       </c>
-      <c r="N2" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="O2" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="P2" s="63" t="inlineStr">
-        <is>
-          <t>WS B - 4</t>
-        </is>
-      </c>
-      <c r="Q2" s="63" t="inlineStr">
-        <is>
-          <t>WS B - 1</t>
-        </is>
-      </c>
-      <c r="R2" s="48" t="inlineStr">
+      <c r="AF11" s="48" t="inlineStr">
         <is>
           <t>MS B - 4</t>
         </is>
       </c>
-      <c r="S2" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="T2" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="U2" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="V2" s="56" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="W2" s="62" t="inlineStr">
-        <is>
-          <t>WD A - 4</t>
-        </is>
-      </c>
-      <c r="X2" s="62" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="Y2" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="Z2" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="AA2" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="AB2" s="57" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="AC2" s="52" t="inlineStr">
+      <c r="AG11" s="62" t="inlineStr">
+        <is>
+          <t>WD A - 2</t>
+        </is>
+      </c>
+      <c r="AH11" s="52" t="inlineStr">
         <is>
           <t>MS A - 4</t>
         </is>
       </c>
-      <c r="AD2" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AE2" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AF2" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="AG2" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="AH2" s="49" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="AI2" s="54" t="inlineStr">
-        <is>
-          <t>WD V - 3</t>
-        </is>
-      </c>
-      <c r="AJ2" s="51" t="inlineStr">
-        <is>
-          <t>MD V - 4</t>
-        </is>
-      </c>
-      <c r="AK2" s="51" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="AL2" s="53" t="inlineStr">
-        <is>
-          <t>WS V - 3</t>
-        </is>
-      </c>
-      <c r="AM2" s="53" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="AN2" s="55" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="AO2" s="55" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="AP2" s="55" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" s="65" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="C3" s="66" t="inlineStr">
-        <is>
-          <t>WD C - 1</t>
-        </is>
-      </c>
-      <c r="D3" s="64" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="E3" s="64" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="F3" s="60" t="inlineStr">
-        <is>
-          <t>WS C - 1</t>
-        </is>
-      </c>
-      <c r="G3" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="H3" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="I3" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="J3" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="K3" s="59" t="inlineStr">
-        <is>
-          <t>XD B - 4</t>
-        </is>
-      </c>
-      <c r="L3" s="59" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="M3" s="61" t="inlineStr">
-        <is>
-          <t>WD B - 2</t>
-        </is>
-      </c>
-      <c r="N3" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="O3" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="P3" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="Q3" s="63" t="inlineStr">
-        <is>
-          <t>WS B - 1</t>
-        </is>
-      </c>
-      <c r="R3" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 4</t>
-        </is>
-      </c>
-      <c r="S3" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="T3" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="U3" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="V3" s="56" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="W3" s="56" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="X3" s="62" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="Y3" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 3</t>
-        </is>
-      </c>
-      <c r="Z3" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="AA3" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="AB3" s="57" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="AC3" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 4</t>
-        </is>
-      </c>
-      <c r="AD3" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AE3" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AF3" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="AG3" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="AH3" s="49" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="AI3" s="54" t="inlineStr">
+      <c r="AI11" s="51" t="inlineStr">
+        <is>
+          <t>MD V - 3</t>
+        </is>
+      </c>
+      <c r="AJ11" s="65" t="inlineStr">
+        <is>
+          <t>XD C - 4</t>
+        </is>
+      </c>
+      <c r="AK11" s="64" t="inlineStr">
+        <is>
+          <t>MD C - 5</t>
+        </is>
+      </c>
+      <c r="AL11" s="61" t="inlineStr">
+        <is>
+          <t>WD B - 4</t>
+        </is>
+      </c>
+      <c r="AM11" s="48" t="inlineStr">
+        <is>
+          <t>MS B - 6</t>
+        </is>
+      </c>
+      <c r="AN11" s="50" t="inlineStr">
+        <is>
+          <t>MD A - 5</t>
+        </is>
+      </c>
+      <c r="AO11" s="54" t="inlineStr">
         <is>
           <t>WD V - 4</t>
-        </is>
-      </c>
-      <c r="AJ3" s="51" t="inlineStr">
-        <is>
-          <t>MD V - 5</t>
-        </is>
-      </c>
-      <c r="AK3" s="51" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="AL3" s="53" t="inlineStr">
-        <is>
-          <t>WS V - 3</t>
-        </is>
-      </c>
-      <c r="AM3" s="53" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="AN3" s="55" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-      <c r="AO3" s="55" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-      <c r="AP3" s="55" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" s="65" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="C4" s="66" t="inlineStr">
-        <is>
-          <t>WD C - 2</t>
-        </is>
-      </c>
-      <c r="D4" s="64" t="inlineStr">
-        <is>
-          <t>MD C - 3</t>
-        </is>
-      </c>
-      <c r="E4" s="64" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="F4" s="60" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="G4" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="H4" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="I4" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="J4" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="K4" s="59" t="inlineStr">
-        <is>
-          <t>XD B - 4</t>
-        </is>
-      </c>
-      <c r="L4" s="59" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="M4" s="61" t="inlineStr">
-        <is>
-          <t>WD B - 3</t>
-        </is>
-      </c>
-      <c r="N4" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="O4" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="P4" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="Q4" s="63" t="inlineStr">
-        <is>
-          <t>WS B - 1</t>
-        </is>
-      </c>
-      <c r="R4" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 4</t>
-        </is>
-      </c>
-      <c r="S4" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="T4" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="U4" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="V4" s="56" t="inlineStr">
-        <is>
-          <t>XD A - 3</t>
-        </is>
-      </c>
-      <c r="W4" s="56" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="X4" s="62" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="Y4" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 3</t>
-        </is>
-      </c>
-      <c r="Z4" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="AA4" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="AB4" s="57" t="inlineStr">
-        <is>
-          <t>WS A - 2</t>
-        </is>
-      </c>
-      <c r="AC4" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 5</t>
-        </is>
-      </c>
-      <c r="AD4" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AE4" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AF4" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="AG4" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="AH4" s="49" t="inlineStr">
-        <is>
-          <t>XD V - 3</t>
-        </is>
-      </c>
-      <c r="AI4" s="49" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="AJ4" s="54" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="AK4" s="51" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="AL4" s="53" t="inlineStr">
-        <is>
-          <t>WS V - 3</t>
-        </is>
-      </c>
-      <c r="AM4" s="53" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="AN4" s="55" t="inlineStr">
-        <is>
-          <t>MS V - 3</t>
-        </is>
-      </c>
-      <c r="AO4" s="55" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="65" t="inlineStr">
-        <is>
-          <t>XD C - 2</t>
-        </is>
-      </c>
-      <c r="C5" s="66" t="inlineStr">
-        <is>
-          <t>WD C - 2</t>
-        </is>
-      </c>
-      <c r="D5" s="64" t="inlineStr">
-        <is>
-          <t>MD C - 3</t>
-        </is>
-      </c>
-      <c r="E5" s="64" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="F5" s="60" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="G5" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 4</t>
-        </is>
-      </c>
-      <c r="H5" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="I5" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="J5" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="K5" s="59" t="inlineStr">
-        <is>
-          <t>XD B - 5</t>
-        </is>
-      </c>
-      <c r="L5" s="59" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="M5" s="61" t="inlineStr">
-        <is>
-          <t>WD B - 3</t>
-        </is>
-      </c>
-      <c r="N5" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 3</t>
-        </is>
-      </c>
-      <c r="O5" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="P5" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="Q5" s="63" t="inlineStr">
-        <is>
-          <t>WS B - 1</t>
-        </is>
-      </c>
-      <c r="R5" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 4</t>
-        </is>
-      </c>
-      <c r="S5" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="T5" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="U5" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="V5" s="56" t="inlineStr">
-        <is>
-          <t>XD A - 3</t>
-        </is>
-      </c>
-      <c r="W5" s="56" t="inlineStr">
-        <is>
-          <t>XD A - 1</t>
-        </is>
-      </c>
-      <c r="X5" s="62" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="Y5" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 3</t>
-        </is>
-      </c>
-      <c r="Z5" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="AA5" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="AB5" s="57" t="inlineStr">
-        <is>
-          <t>WS A - 2</t>
-        </is>
-      </c>
-      <c r="AC5" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 5</t>
-        </is>
-      </c>
-      <c r="AD5" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AE5" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AF5" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="AG5" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="AH5" s="49" t="inlineStr">
-        <is>
-          <t>XD V - 3</t>
-        </is>
-      </c>
-      <c r="AI5" s="49" t="inlineStr">
-        <is>
-          <t>XD V - 1</t>
-        </is>
-      </c>
-      <c r="AJ5" s="54" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="AK5" s="51" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="AL5" s="53" t="inlineStr">
-        <is>
-          <t>WS V - 4</t>
-        </is>
-      </c>
-      <c r="AM5" s="53" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="AN5" s="55" t="inlineStr">
-        <is>
-          <t>MS V - 3</t>
-        </is>
-      </c>
-      <c r="AO5" s="55" t="inlineStr">
-        <is>
-          <t>MS V - 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="65" t="inlineStr">
-        <is>
-          <t>XD C - 2</t>
-        </is>
-      </c>
-      <c r="C6" s="66" t="inlineStr">
-        <is>
-          <t>WD C - 3</t>
-        </is>
-      </c>
-      <c r="D6" s="64" t="inlineStr">
-        <is>
-          <t>MD C - 3</t>
-        </is>
-      </c>
-      <c r="E6" s="64" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="F6" s="60" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="G6" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 4</t>
-        </is>
-      </c>
-      <c r="H6" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="I6" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="J6" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="K6" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="L6" s="59" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="M6" s="61" t="inlineStr">
-        <is>
-          <t>WD B - 4</t>
-        </is>
-      </c>
-      <c r="N6" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 4</t>
-        </is>
-      </c>
-      <c r="O6" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="P6" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="Q6" s="63" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="R6" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 5</t>
-        </is>
-      </c>
-      <c r="S6" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="T6" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="U6" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="V6" s="56" t="inlineStr">
-        <is>
-          <t>XD A - 3</t>
-        </is>
-      </c>
-      <c r="W6" s="56" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="X6" s="62" t="inlineStr">
-        <is>
-          <t>WD A - 2</t>
-        </is>
-      </c>
-      <c r="Y6" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 3</t>
-        </is>
-      </c>
-      <c r="Z6" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="AA6" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="AB6" s="57" t="inlineStr">
-        <is>
-          <t>WS A - 2</t>
-        </is>
-      </c>
-      <c r="AC6" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 6</t>
-        </is>
-      </c>
-      <c r="AD6" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AE6" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AF6" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AG6" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="AH6" s="49" t="inlineStr">
-        <is>
-          <t>XD V - 3</t>
-        </is>
-      </c>
-      <c r="AI6" s="49" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="AJ6" s="54" t="inlineStr">
-        <is>
-          <t>WD V - 1</t>
-        </is>
-      </c>
-      <c r="AK6" s="51" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="AL6" s="53" t="inlineStr">
-        <is>
-          <t>WS V - 4</t>
-        </is>
-      </c>
-      <c r="AM6" s="53" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="AN6" s="55" t="inlineStr">
-        <is>
-          <t>MS V - 3</t>
-        </is>
-      </c>
-      <c r="AO6" s="55" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="65" t="inlineStr">
-        <is>
-          <t>XD C - 2</t>
-        </is>
-      </c>
-      <c r="C7" s="65" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="D7" s="64" t="inlineStr">
-        <is>
-          <t>MD C - 3</t>
-        </is>
-      </c>
-      <c r="E7" s="64" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="F7" s="60" t="inlineStr">
-        <is>
-          <t>WS C - 2</t>
-        </is>
-      </c>
-      <c r="G7" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 4</t>
-        </is>
-      </c>
-      <c r="H7" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="I7" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="J7" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="K7" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="L7" s="59" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="M7" s="59" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="N7" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 4</t>
-        </is>
-      </c>
-      <c r="O7" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="P7" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="Q7" s="63" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="R7" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 5</t>
-        </is>
-      </c>
-      <c r="S7" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="T7" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="U7" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="V7" s="56" t="inlineStr">
-        <is>
-          <t>XD A - 3</t>
-        </is>
-      </c>
-      <c r="W7" s="56" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="X7" s="62" t="inlineStr">
-        <is>
-          <t>WD A - 2</t>
-        </is>
-      </c>
-      <c r="Y7" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 4</t>
-        </is>
-      </c>
-      <c r="Z7" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="AA7" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="AB7" s="57" t="inlineStr">
-        <is>
-          <t>WS A - 2</t>
-        </is>
-      </c>
-      <c r="AC7" s="57" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="AD7" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AE7" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AF7" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AG7" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="AH7" s="49" t="inlineStr">
-        <is>
-          <t>XD V - 3</t>
-        </is>
-      </c>
-      <c r="AI7" s="49" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="AJ7" s="54" t="inlineStr">
-        <is>
-          <t>WD V - 2</t>
-        </is>
-      </c>
-      <c r="AK7" s="51" t="inlineStr">
-        <is>
-          <t>MD V - 3</t>
-        </is>
-      </c>
-      <c r="AL7" s="53" t="inlineStr">
-        <is>
-          <t>WS V - 5</t>
-        </is>
-      </c>
-      <c r="AM7" s="53" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="AN7" s="55" t="inlineStr">
-        <is>
-          <t>MS V - 3</t>
-        </is>
-      </c>
-      <c r="AO7" s="55" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="65" t="inlineStr">
-        <is>
-          <t>XD C - 2</t>
-        </is>
-      </c>
-      <c r="C8" s="65" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="D8" s="64" t="inlineStr">
-        <is>
-          <t>MD C - 4</t>
-        </is>
-      </c>
-      <c r="E8" s="64" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="F8" s="60" t="inlineStr">
-        <is>
-          <t>WS C - 3</t>
-        </is>
-      </c>
-      <c r="G8" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 4</t>
-        </is>
-      </c>
-      <c r="H8" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="I8" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="J8" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="K8" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="L8" s="59" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="M8" s="59" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="N8" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 5</t>
-        </is>
-      </c>
-      <c r="O8" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="P8" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="Q8" s="63" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="R8" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 6</t>
-        </is>
-      </c>
-      <c r="S8" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="T8" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="U8" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="V8" s="56" t="inlineStr">
-        <is>
-          <t>XD A - 4</t>
-        </is>
-      </c>
-      <c r="W8" s="56" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="X8" s="62" t="inlineStr">
-        <is>
-          <t>WD A - 2</t>
-        </is>
-      </c>
-      <c r="Y8" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 4</t>
-        </is>
-      </c>
-      <c r="Z8" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="AA8" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="AB8" s="57" t="inlineStr">
-        <is>
-          <t>WS A - 3</t>
-        </is>
-      </c>
-      <c r="AC8" s="57" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="AD8" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AE8" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AF8" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AG8" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="AH8" s="49" t="inlineStr">
-        <is>
-          <t>XD V - 4</t>
-        </is>
-      </c>
-      <c r="AI8" s="49" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="AJ8" s="54" t="inlineStr">
-        <is>
-          <t>WD V - 2</t>
-        </is>
-      </c>
-      <c r="AK8" s="51" t="inlineStr">
-        <is>
-          <t>MD V - 3</t>
-        </is>
-      </c>
-      <c r="AL8" s="51" t="inlineStr">
-        <is>
-          <t>MD V - 1</t>
-        </is>
-      </c>
-      <c r="AM8" s="53" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="AN8" s="55" t="inlineStr">
-        <is>
-          <t>MS V - 4</t>
-        </is>
-      </c>
-      <c r="AO8" s="55" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="65" t="inlineStr">
-        <is>
-          <t>XD C - 3</t>
-        </is>
-      </c>
-      <c r="C9" s="65" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="D9" s="64" t="inlineStr">
-        <is>
-          <t>MD C - 4</t>
-        </is>
-      </c>
-      <c r="E9" s="64" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="F9" s="60" t="inlineStr">
-        <is>
-          <t>WS C - 3</t>
-        </is>
-      </c>
-      <c r="G9" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 5</t>
-        </is>
-      </c>
-      <c r="H9" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="I9" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="J9" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="K9" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="L9" s="59" t="inlineStr">
-        <is>
-          <t>XD B - 3</t>
-        </is>
-      </c>
-      <c r="M9" s="59" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="N9" s="61" t="inlineStr">
-        <is>
-          <t>WD B - 1</t>
-        </is>
-      </c>
-      <c r="O9" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="P9" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="Q9" s="63" t="inlineStr">
-        <is>
-          <t>WS B - 2</t>
-        </is>
-      </c>
-      <c r="R9" s="63" t="inlineStr">
-        <is>
-          <t>WS B - 1</t>
-        </is>
-      </c>
-      <c r="S9" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="T9" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="U9" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="V9" s="56" t="inlineStr">
-        <is>
-          <t>XD A - 4</t>
-        </is>
-      </c>
-      <c r="W9" s="56" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="X9" s="62" t="inlineStr">
-        <is>
-          <t>WD A - 2</t>
-        </is>
-      </c>
-      <c r="Y9" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 5</t>
-        </is>
-      </c>
-      <c r="Z9" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="AA9" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="AB9" s="57" t="inlineStr">
-        <is>
-          <t>WS A - 3</t>
-        </is>
-      </c>
-      <c r="AC9" s="57" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="AD9" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 3</t>
-        </is>
-      </c>
-      <c r="AE9" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AF9" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AG9" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="AH9" s="49" t="inlineStr">
-        <is>
-          <t>XD V - 4</t>
-        </is>
-      </c>
-      <c r="AI9" s="49" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="AJ9" s="54" t="inlineStr">
-        <is>
-          <t>WD V - 2</t>
-        </is>
-      </c>
-      <c r="AK9" s="51" t="inlineStr">
-        <is>
-          <t>MD V - 3</t>
-        </is>
-      </c>
-      <c r="AL9" s="51" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="AM9" s="53" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="AN9" s="55" t="inlineStr">
-        <is>
-          <t>MS V - 4</t>
-        </is>
-      </c>
-      <c r="AO9" s="55" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="65" t="inlineStr">
-        <is>
-          <t>XD C - 3</t>
-        </is>
-      </c>
-      <c r="C10" s="65" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="D10" s="64" t="inlineStr">
-        <is>
-          <t>MD C - 5</t>
-        </is>
-      </c>
-      <c r="E10" s="64" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="F10" s="60" t="inlineStr">
-        <is>
-          <t>WS C - 4</t>
-        </is>
-      </c>
-      <c r="G10" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 5</t>
-        </is>
-      </c>
-      <c r="H10" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="I10" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="J10" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="K10" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="L10" s="59" t="inlineStr">
-        <is>
-          <t>XD B - 3</t>
-        </is>
-      </c>
-      <c r="M10" s="59" t="inlineStr">
-        <is>
-          <t>XD B - 1</t>
-        </is>
-      </c>
-      <c r="N10" s="61" t="inlineStr">
-        <is>
-          <t>WD B - 2</t>
-        </is>
-      </c>
-      <c r="O10" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="P10" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="Q10" s="63" t="inlineStr">
-        <is>
-          <t>WS B - 3</t>
-        </is>
-      </c>
-      <c r="R10" s="63" t="inlineStr">
-        <is>
-          <t>WS B - 1</t>
-        </is>
-      </c>
-      <c r="S10" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="T10" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="U10" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="V10" s="56" t="inlineStr">
-        <is>
-          <t>XD A - 5</t>
-        </is>
-      </c>
-      <c r="W10" s="56" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="X10" s="62" t="inlineStr">
-        <is>
-          <t>WD A - 3</t>
-        </is>
-      </c>
-      <c r="Y10" s="62" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="Z10" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="AA10" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="AB10" s="57" t="inlineStr">
-        <is>
-          <t>WS A - 4</t>
-        </is>
-      </c>
-      <c r="AC10" s="57" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="AD10" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 4</t>
-        </is>
-      </c>
-      <c r="AE10" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AF10" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AG10" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="AH10" s="49" t="inlineStr">
-        <is>
-          <t>XD V - 5</t>
-        </is>
-      </c>
-      <c r="AI10" s="49" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="AJ10" s="54" t="inlineStr">
-        <is>
-          <t>WD V - 2</t>
-        </is>
-      </c>
-      <c r="AK10" s="51" t="inlineStr">
-        <is>
-          <t>MD V - 3</t>
-        </is>
-      </c>
-      <c r="AL10" s="51" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="AM10" s="53" t="inlineStr">
-        <is>
-          <t>WS V - 2</t>
-        </is>
-      </c>
-      <c r="AN10" s="55" t="inlineStr">
-        <is>
-          <t>MS V - 5</t>
-        </is>
-      </c>
-      <c r="AO10" s="55" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="65" t="inlineStr">
-        <is>
-          <t>XD C - 4</t>
-        </is>
-      </c>
-      <c r="C11" s="65" t="inlineStr">
-        <is>
-          <t>XD C - 1</t>
-        </is>
-      </c>
-      <c r="D11" s="66" t="inlineStr">
-        <is>
-          <t>WD C - 1</t>
-        </is>
-      </c>
-      <c r="E11" s="64" t="inlineStr">
-        <is>
-          <t>MD C - 2</t>
-        </is>
-      </c>
-      <c r="F11" s="64" t="inlineStr">
-        <is>
-          <t>MD C - 1</t>
-        </is>
-      </c>
-      <c r="G11" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 6</t>
-        </is>
-      </c>
-      <c r="H11" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 3</t>
-        </is>
-      </c>
-      <c r="I11" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="J11" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 2</t>
-        </is>
-      </c>
-      <c r="K11" s="47" t="inlineStr">
-        <is>
-          <t>MS C - 1</t>
-        </is>
-      </c>
-      <c r="L11" s="59" t="inlineStr">
-        <is>
-          <t>XD B - 3</t>
-        </is>
-      </c>
-      <c r="M11" s="59" t="inlineStr">
-        <is>
-          <t>XD B - 2</t>
-        </is>
-      </c>
-      <c r="N11" s="61" t="inlineStr">
-        <is>
-          <t>WD B - 2</t>
-        </is>
-      </c>
-      <c r="O11" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 2</t>
-        </is>
-      </c>
-      <c r="P11" s="58" t="inlineStr">
-        <is>
-          <t>MD B - 1</t>
-        </is>
-      </c>
-      <c r="Q11" s="63" t="inlineStr">
-        <is>
-          <t>WS B - 3</t>
-        </is>
-      </c>
-      <c r="R11" s="63" t="inlineStr">
-        <is>
-          <t>WS B - 1</t>
-        </is>
-      </c>
-      <c r="S11" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 3</t>
-        </is>
-      </c>
-      <c r="T11" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="U11" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 2</t>
-        </is>
-      </c>
-      <c r="V11" s="48" t="inlineStr">
-        <is>
-          <t>MS B - 1</t>
-        </is>
-      </c>
-      <c r="W11" s="56" t="inlineStr">
-        <is>
-          <t>XD A - 2</t>
-        </is>
-      </c>
-      <c r="X11" s="62" t="inlineStr">
-        <is>
-          <t>WD A - 3</t>
-        </is>
-      </c>
-      <c r="Y11" s="62" t="inlineStr">
-        <is>
-          <t>WD A - 1</t>
-        </is>
-      </c>
-      <c r="Z11" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 2</t>
-        </is>
-      </c>
-      <c r="AA11" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="AB11" s="50" t="inlineStr">
-        <is>
-          <t>MD A - 1</t>
-        </is>
-      </c>
-      <c r="AC11" s="57" t="inlineStr">
-        <is>
-          <t>WS A - 1</t>
-        </is>
-      </c>
-      <c r="AD11" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 4</t>
-        </is>
-      </c>
-      <c r="AE11" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AF11" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 2</t>
-        </is>
-      </c>
-      <c r="AG11" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="AH11" s="52" t="inlineStr">
-        <is>
-          <t>MS A - 1</t>
-        </is>
-      </c>
-      <c r="AI11" s="49" t="inlineStr">
-        <is>
-          <t>XD V - 2</t>
-        </is>
-      </c>
-      <c r="AJ11" s="54" t="inlineStr">
-        <is>
-          <t>WD V - 3</t>
-        </is>
-      </c>
-      <c r="AK11" s="51" t="inlineStr">
-        <is>
-          <t>MD V - 4</t>
-        </is>
-      </c>
-      <c r="AL11" s="51" t="inlineStr">
-        <is>
-          <t>MD V - 2</t>
-        </is>
-      </c>
-      <c r="AM11" s="53" t="inlineStr">
-        <is>
-          <t>WS V - 3</t>
-        </is>
-      </c>
-      <c r="AN11" s="53" t="inlineStr">
-        <is>
-          <t>WS V - 1</t>
-        </is>
-      </c>
-      <c r="AO11" s="55" t="inlineStr">
-        <is>
-          <t>MS V - 2</t>
         </is>
       </c>
     </row>

</xml_diff>